<commit_message>
Finished processing of various test splits
</commit_message>
<xml_diff>
--- a/Visualization/Individual Calix Regression Organized.xlsx
+++ b/Visualization/Individual Calix Regression Organized.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffreyvanhumbeck/Documents/GitHub/Calixarenes/Visualization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F01B03FE-D73D-864A-B18D-D0D455F70208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8672D106-353A-C940-9D0A-2FDC6A2B01EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37980" yWindow="1780" windowWidth="29480" windowHeight="19880" xr2:uid="{FEEF7F71-20B1-1443-B210-33355AD765BD}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="10000" windowHeight="18740" xr2:uid="{FEEF7F71-20B1-1443-B210-33355AD765BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -3672,83 +3672,83 @@
         <v>40</v>
       </c>
       <c r="B47" s="24">
-        <f>MEDIAN(B3:B22,B37:B42,B44:B45)</f>
+        <f t="shared" ref="B47:U47" si="0">MEDIAN(B3:B22,B37:B42,B44:B45)</f>
         <v>0.51550000000000007</v>
       </c>
       <c r="C47" s="25">
-        <f>MEDIAN(C3:C22,C37:C42,C44:C45)</f>
+        <f t="shared" si="0"/>
         <v>0.81850000000000001</v>
       </c>
       <c r="D47" s="26">
-        <f>MEDIAN(D3:D22,D37:D42,D44:D45)</f>
+        <f t="shared" si="0"/>
         <v>0.437</v>
       </c>
       <c r="E47" s="27">
-        <f>MEDIAN(E3:E22,E37:E42,E44:E45)</f>
+        <f t="shared" si="0"/>
         <v>0.82450000000000001</v>
       </c>
       <c r="F47" s="24">
-        <f>MEDIAN(F3:F22,F37:F42,F44:F45)</f>
+        <f t="shared" si="0"/>
         <v>0.48649999999999999</v>
       </c>
       <c r="G47" s="25">
-        <f>MEDIAN(G3:G22,G37:G42,G44:G45)</f>
+        <f t="shared" si="0"/>
         <v>0.69899999999999995</v>
       </c>
       <c r="H47" s="26">
-        <f>MEDIAN(H3:H22,H37:H42,H44:H45)</f>
+        <f t="shared" si="0"/>
         <v>-6.7449999999999996E-2</v>
       </c>
       <c r="I47" s="27">
-        <f>MEDIAN(I3:I22,I37:I42,I44:I45)</f>
+        <f t="shared" si="0"/>
         <v>0.85230000000000006</v>
       </c>
       <c r="J47" s="24">
-        <f>MEDIAN(J3:J22,J37:J42,J44:J45)</f>
+        <f t="shared" si="0"/>
         <v>-0.28295000000000003</v>
       </c>
       <c r="K47" s="25">
-        <f>MEDIAN(K3:K22,K37:K42,K44:K45)</f>
+        <f t="shared" si="0"/>
         <v>0.61945000000000006</v>
       </c>
       <c r="L47" s="26">
-        <f>MEDIAN(L3:L22,L37:L42,L44:L45)</f>
+        <f t="shared" si="0"/>
         <v>-9.0999999999999998E-2</v>
       </c>
       <c r="M47" s="27">
-        <f>MEDIAN(M3:M22,M37:M42,M44:M45)</f>
+        <f t="shared" si="0"/>
         <v>0.8589</v>
       </c>
       <c r="N47" s="24">
-        <f>MEDIAN(N3:N22,N37:N42,N44:N45)</f>
+        <f t="shared" si="0"/>
         <v>0.65</v>
       </c>
       <c r="O47" s="25">
-        <f>MEDIAN(O3:O22,O37:O42,O44:O45)</f>
+        <f t="shared" si="0"/>
         <v>0.79</v>
       </c>
       <c r="P47" s="26">
-        <f>MEDIAN(P3:P22,P37:P42,P44:P45)</f>
+        <f t="shared" si="0"/>
         <v>0.08</v>
       </c>
       <c r="Q47" s="27">
-        <f>MEDIAN(Q3:Q22,Q37:Q42,Q44:Q45)</f>
+        <f t="shared" si="0"/>
         <v>0.84</v>
       </c>
       <c r="R47" s="24">
-        <f>MEDIAN(R3:R22,R37:R42,R44:R45)</f>
+        <f t="shared" si="0"/>
         <v>0.82000000000000006</v>
       </c>
       <c r="S47" s="25">
-        <f>MEDIAN(S3:S22,S37:S42,S44:S45)</f>
+        <f t="shared" si="0"/>
         <v>0.92500000000000004</v>
       </c>
       <c r="T47" s="26">
-        <f>MEDIAN(T3:T22,T37:T42,T44:T45)</f>
+        <f t="shared" si="0"/>
         <v>0.16</v>
       </c>
       <c r="U47" s="27">
-        <f>MEDIAN(U3:U22,U37:U42,U44:U45)</f>
+        <f t="shared" si="0"/>
         <v>0.84</v>
       </c>
     </row>
@@ -3757,67 +3757,67 @@
         <v>41</v>
       </c>
       <c r="B48" s="24">
-        <f t="shared" ref="B48:I48" si="0">MEDIAN(B24:B27,B29:B30,B32:B35)</f>
+        <f t="shared" ref="B48:I48" si="1">MEDIAN(B24:B27,B29:B30,B32:B35)</f>
         <v>-0.63900000000000001</v>
       </c>
       <c r="C48" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-4.6499999999999986E-2</v>
       </c>
       <c r="D48" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.86299999999999999</v>
       </c>
       <c r="E48" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.20250000000000001</v>
       </c>
       <c r="F48" s="24">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.75350000000000006</v>
       </c>
       <c r="G48" s="25">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.30449999999999999</v>
       </c>
       <c r="H48" s="26">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.85759999999999992</v>
       </c>
       <c r="I48" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.14845</v>
       </c>
       <c r="J48" s="24">
-        <f t="shared" ref="J48:Q48" si="1">MEDIAN(J24:J27,J29:J30,J32:J35)</f>
+        <f t="shared" ref="J48:Q48" si="2">MEDIAN(J24:J27,J29:J30,J32:J35)</f>
         <v>-1.2199499999999999</v>
       </c>
       <c r="K48" s="25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-0.85140000000000005</v>
       </c>
       <c r="L48" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1.3451</v>
       </c>
       <c r="M48" s="27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1.0453999999999999</v>
       </c>
       <c r="N48" s="24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.33500000000000002</v>
       </c>
       <c r="O48" s="25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-0.21</v>
       </c>
       <c r="P48" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-0.67999999999999994</v>
       </c>
       <c r="Q48" s="27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-0.05</v>
       </c>
       <c r="R48" s="24">
@@ -3829,11 +3829,11 @@
         <v>0.72</v>
       </c>
       <c r="T48" s="26">
-        <f t="shared" ref="T48:U48" si="2">MEDIAN(T24:T27,T29:T30,T32:T35)</f>
+        <f t="shared" ref="T48:U48" si="3">MEDIAN(T24:T27,T29:T30,T32:T35)</f>
         <v>-0.72</v>
       </c>
       <c r="U48" s="27">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-0.15000000000000002</v>
       </c>
     </row>
@@ -5779,67 +5779,67 @@
         <v>40</v>
       </c>
       <c r="B83" s="24">
-        <f>MEDIAN(B52:B71,B73:B78,B80:B81)</f>
+        <f t="shared" ref="B83:M83" si="4">MEDIAN(B52:B71,B73:B78,B80:B81)</f>
         <v>0.63050000000000006</v>
       </c>
       <c r="C83" s="25">
-        <f>MEDIAN(C52:C71,C73:C78,C80:C81)</f>
+        <f t="shared" si="4"/>
         <v>0.85050000000000003</v>
       </c>
       <c r="D83" s="26">
-        <f>MEDIAN(D52:D71,D73:D78,D80:D81)</f>
+        <f t="shared" si="4"/>
         <v>0.6915</v>
       </c>
       <c r="E83" s="27">
-        <f>MEDIAN(E52:E71,E73:E78,E80:E81)</f>
+        <f t="shared" si="4"/>
         <v>0.89100000000000001</v>
       </c>
       <c r="F83" s="24">
-        <f>MEDIAN(F52:F71,F73:F78,F80:F81)</f>
+        <f t="shared" si="4"/>
         <v>0.51800000000000002</v>
       </c>
       <c r="G83" s="25">
-        <f>MEDIAN(G52:G71,G73:G78,G80:G81)</f>
+        <f t="shared" si="4"/>
         <v>0.69750000000000001</v>
       </c>
       <c r="H83" s="26">
-        <f>MEDIAN(H52:H71,H73:H78,H80:H81)</f>
+        <f t="shared" si="4"/>
         <v>0.55449999999999999</v>
       </c>
       <c r="I83" s="27">
-        <f>MEDIAN(I52:I71,I73:I78,I80:I81)</f>
+        <f t="shared" si="4"/>
         <v>0.87450000000000006</v>
       </c>
       <c r="J83" s="24">
-        <f>MEDIAN(J52:J71,J73:J78,J80:J81)</f>
+        <f t="shared" si="4"/>
         <v>-0.1305</v>
       </c>
       <c r="K83" s="25">
-        <f>MEDIAN(K52:K71,K73:K78,K80:K81)</f>
+        <f t="shared" si="4"/>
         <v>0.34599999999999997</v>
       </c>
       <c r="L83" s="26">
-        <f>MEDIAN(L52:L71,L73:L78,L80:L81)</f>
+        <f t="shared" si="4"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="M83" s="27">
-        <f>MEDIAN(M52:M71,M73:M78,M80:M81)</f>
+        <f t="shared" si="4"/>
         <v>0.89700000000000002</v>
       </c>
       <c r="N83" s="24">
-        <f t="shared" ref="N83:Q83" si="3">MEDIAN(N52:N71,N73:N78,N80:N81)</f>
+        <f t="shared" ref="N83:Q83" si="5">MEDIAN(N52:N71,N73:N78,N80:N81)</f>
         <v>0.60499999999999998</v>
       </c>
       <c r="O83" s="25">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.71</v>
       </c>
       <c r="P83" s="26">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>-3.5000000000000003E-2</v>
       </c>
       <c r="Q83" s="27">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>0.89</v>
       </c>
       <c r="R83" s="24">

</xml_diff>

<commit_message>
Final plots for draft
</commit_message>
<xml_diff>
--- a/Visualization/Individual Calix Regression Organized.xlsx
+++ b/Visualization/Individual Calix Regression Organized.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffreyvanhumbeck/Documents/GitHub/Calixarenes/Visualization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8672D106-353A-C940-9D0A-2FDC6A2B01EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD1E0D7-3579-2344-B750-C632420D6041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="10000" windowHeight="18740" xr2:uid="{FEEF7F71-20B1-1443-B210-33355AD765BD}"/>
+    <workbookView xWindow="15180" yWindow="1020" windowWidth="20660" windowHeight="17560" xr2:uid="{FEEF7F71-20B1-1443-B210-33355AD765BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1098,10 +1098,10 @@
         <v>0.91210000000000002</v>
       </c>
       <c r="J3" s="18">
-        <v>0.93810000000000004</v>
+        <v>0.94</v>
       </c>
       <c r="K3" s="16">
-        <v>0.90569999999999995</v>
+        <v>0.91</v>
       </c>
       <c r="L3" s="13">
         <v>0.90600000000000003</v>
@@ -1163,10 +1163,10 @@
         <v>0.95740000000000003</v>
       </c>
       <c r="J4" s="18">
-        <v>0.77110000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="K4" s="16">
-        <v>0.53310000000000002</v>
+        <v>0.53</v>
       </c>
       <c r="L4" s="13">
         <v>0.79330000000000001</v>
@@ -1228,10 +1228,10 @@
         <v>0.92720000000000002</v>
       </c>
       <c r="J5" s="18">
-        <v>0.80830000000000002</v>
+        <v>0.81</v>
       </c>
       <c r="K5" s="16">
-        <v>0.624</v>
+        <v>0.62</v>
       </c>
       <c r="L5" s="13">
         <v>0.7601</v>
@@ -1293,10 +1293,10 @@
         <v>0.91620000000000001</v>
       </c>
       <c r="J6" s="18">
-        <v>0.82550000000000001</v>
+        <v>0.75</v>
       </c>
       <c r="K6" s="16">
-        <v>0.48459999999999998</v>
+        <v>0.83</v>
       </c>
       <c r="L6" s="13">
         <v>0.72750000000000004</v>
@@ -1358,10 +1358,10 @@
         <v>0.71260000000000001</v>
       </c>
       <c r="J7" s="18">
-        <v>0.16969999999999999</v>
+        <v>0.17</v>
       </c>
       <c r="K7" s="16">
-        <v>0.77569999999999995</v>
+        <v>0.78</v>
       </c>
       <c r="L7" s="13">
         <v>0.81169999999999998</v>
@@ -1423,10 +1423,10 @@
         <v>0.49830000000000002</v>
       </c>
       <c r="J8" s="18">
-        <v>0.21590000000000001</v>
+        <v>0.22</v>
       </c>
       <c r="K8" s="16">
-        <v>0.56589999999999996</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="L8" s="13">
         <v>-0.15359999999999999</v>
@@ -1488,10 +1488,10 @@
         <v>0.70679999999999998</v>
       </c>
       <c r="J9" s="18">
-        <v>-1.2966</v>
+        <v>-1.3</v>
       </c>
       <c r="K9" s="16">
-        <v>-0.19370000000000001</v>
+        <v>-0.19</v>
       </c>
       <c r="L9" s="13">
         <v>-1.6005</v>
@@ -1553,10 +1553,10 @@
         <v>0.63449999999999995</v>
       </c>
       <c r="J10" s="18">
-        <v>-4.7000000000000002E-3</v>
+        <v>0</v>
       </c>
       <c r="K10" s="16">
-        <v>-5.3239000000000001</v>
+        <v>-5.32</v>
       </c>
       <c r="L10" s="13">
         <v>-1.4079999999999999</v>
@@ -1618,10 +1618,10 @@
         <v>0.51759999999999995</v>
       </c>
       <c r="J11" s="18">
-        <v>-0.4672</v>
+        <v>-0.47</v>
       </c>
       <c r="K11" s="16">
-        <v>-7.5967000000000002</v>
+        <v>-7.6</v>
       </c>
       <c r="L11" s="13">
         <v>0.64929999999999999</v>
@@ -1683,10 +1683,10 @@
         <v>0.7</v>
       </c>
       <c r="J12" s="18">
-        <v>-9.8699999999999996E-2</v>
+        <v>-0.1</v>
       </c>
       <c r="K12" s="16">
-        <v>0.87050000000000005</v>
+        <v>0.87</v>
       </c>
       <c r="L12" s="13">
         <v>-0.1983</v>
@@ -1748,10 +1748,10 @@
         <v>0.78449999999999998</v>
       </c>
       <c r="J13" s="18">
-        <v>-0.54649999999999999</v>
+        <v>-0.55000000000000004</v>
       </c>
       <c r="K13" s="16">
-        <v>0.6149</v>
+        <v>0.61</v>
       </c>
       <c r="L13" s="13">
         <v>-0.63109999999999999</v>
@@ -1813,10 +1813,10 @@
         <v>0.35249999999999998</v>
       </c>
       <c r="J14" s="18">
-        <v>-0.69510000000000005</v>
+        <v>-0.42</v>
       </c>
       <c r="K14" s="16">
-        <v>2.4400000000000002E-2</v>
+        <v>0.05</v>
       </c>
       <c r="L14" s="13">
         <v>-0.31519999999999998</v>
@@ -1878,10 +1878,10 @@
         <v>0.87939999999999996</v>
       </c>
       <c r="J15" s="18">
-        <v>-1.5590999999999999</v>
+        <v>-1.56</v>
       </c>
       <c r="K15" s="16">
-        <v>0.94920000000000004</v>
+        <v>0.95</v>
       </c>
       <c r="L15" s="13">
         <v>-0.86050000000000004</v>
@@ -1943,10 +1943,10 @@
         <v>0.87939999999999996</v>
       </c>
       <c r="J16" s="18">
-        <v>-0.68740000000000001</v>
+        <v>-0.69</v>
       </c>
       <c r="K16" s="16">
-        <v>0.88470000000000004</v>
+        <v>0.88</v>
       </c>
       <c r="L16" s="13">
         <v>-0.65069999999999995</v>
@@ -2008,10 +2008,10 @@
         <v>0.96179999999999999</v>
       </c>
       <c r="J17" s="18">
-        <v>0.128</v>
+        <v>0.13</v>
       </c>
       <c r="K17" s="16">
-        <v>-0.21679999999999999</v>
+        <v>-0.22</v>
       </c>
       <c r="L17" s="13">
         <v>0.50319999999999998</v>
@@ -2073,10 +2073,10 @@
         <v>0.95020000000000004</v>
       </c>
       <c r="J18" s="18">
-        <v>0.95730000000000004</v>
+        <v>0.96</v>
       </c>
       <c r="K18" s="16">
-        <v>0.98280000000000001</v>
+        <v>0.98</v>
       </c>
       <c r="L18" s="13">
         <v>0.88529999999999998</v>
@@ -2138,10 +2138,10 @@
         <v>0.82520000000000004</v>
       </c>
       <c r="J19" s="18">
-        <v>0.64339999999999997</v>
+        <v>0.64</v>
       </c>
       <c r="K19" s="16">
-        <v>0.39340000000000003</v>
+        <v>0.39</v>
       </c>
       <c r="L19" s="13">
         <v>0.70709999999999995</v>
@@ -2203,10 +2203,10 @@
         <v>0.91069999999999995</v>
       </c>
       <c r="J20" s="18">
-        <v>-3.0653999999999999</v>
+        <v>-3.07</v>
       </c>
       <c r="K20" s="16">
-        <v>0.89249999999999996</v>
+        <v>0.89</v>
       </c>
       <c r="L20" s="13">
         <v>-1.3620000000000001</v>
@@ -2268,10 +2268,10 @@
         <v>0.67900000000000005</v>
       </c>
       <c r="J21" s="18">
-        <v>0.36320000000000002</v>
+        <v>0.36</v>
       </c>
       <c r="K21" s="16">
-        <v>0.71870000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="L21" s="13">
         <v>0.77310000000000001</v>
@@ -2333,10 +2333,10 @@
         <v>0.91900000000000004</v>
       </c>
       <c r="J22" s="18">
-        <v>0.74009999999999998</v>
+        <v>0.74</v>
       </c>
       <c r="K22" s="16">
-        <v>0.76739999999999997</v>
+        <v>0.77</v>
       </c>
       <c r="L22" s="13">
         <v>6.7500000000000004E-2</v>
@@ -2420,10 +2420,10 @@
         <v>-0.3463</v>
       </c>
       <c r="J24" s="18">
-        <v>-1.1435</v>
+        <v>-1.1399999999999999</v>
       </c>
       <c r="K24" s="16">
-        <v>-7.6351000000000004</v>
+        <v>-7.64</v>
       </c>
       <c r="L24" s="13">
         <v>-1.2584</v>
@@ -2485,10 +2485,10 @@
         <v>0.47420000000000001</v>
       </c>
       <c r="J25" s="18">
-        <v>-1.8652</v>
+        <v>-1.87</v>
       </c>
       <c r="K25" s="16">
-        <v>-0.18809999999999999</v>
+        <v>-0.19</v>
       </c>
       <c r="L25" s="13">
         <v>-1.9758</v>
@@ -2550,10 +2550,10 @@
         <v>-0.15479999999999999</v>
       </c>
       <c r="J26" s="18">
-        <v>-3.7723</v>
+        <v>-3.77</v>
       </c>
       <c r="K26" s="16">
-        <v>-17.5456</v>
+        <v>-17.55</v>
       </c>
       <c r="L26" s="13">
         <v>-1.397</v>
@@ -2615,10 +2615,10 @@
         <v>0.41049999999999998</v>
       </c>
       <c r="J27" s="18">
-        <v>-22.1419</v>
+        <v>-22.14</v>
       </c>
       <c r="K27" s="16">
-        <v>-3.6400000000000002E-2</v>
+        <v>-0.04</v>
       </c>
       <c r="L27" s="13">
         <v>-39.194499999999998</v>
@@ -2702,10 +2702,10 @@
         <v>-0.1421</v>
       </c>
       <c r="J29" s="18">
-        <v>-0.23830000000000001</v>
+        <v>-0.24</v>
       </c>
       <c r="K29" s="16">
-        <v>-0.31709999999999999</v>
+        <v>-0.32</v>
       </c>
       <c r="L29" s="13">
         <v>-0.43890000000000001</v>
@@ -2767,10 +2767,10 @@
         <v>-1.242</v>
       </c>
       <c r="J30" s="18">
-        <v>-0.51359999999999995</v>
+        <v>-0.51</v>
       </c>
       <c r="K30" s="16">
-        <v>-2.4342000000000001</v>
+        <v>-2.4300000000000002</v>
       </c>
       <c r="L30" s="13">
         <v>-0.67400000000000004</v>
@@ -2854,10 +2854,10 @@
         <v>0.89739999999999998</v>
       </c>
       <c r="J32" s="18">
-        <v>-0.1719</v>
+        <v>-0.17</v>
       </c>
       <c r="K32" s="16">
-        <v>0.90010000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="L32" s="13">
         <v>-2.7035999999999998</v>
@@ -2919,10 +2919,10 @@
         <v>7.9699999999999993E-2</v>
       </c>
       <c r="J33" s="18">
-        <v>-0.4007</v>
+        <v>-0.4</v>
       </c>
       <c r="K33" s="16">
-        <v>-0.40060000000000001</v>
+        <v>-0.4</v>
       </c>
       <c r="L33" s="13">
         <v>-0.3301</v>
@@ -2984,10 +2984,10 @@
         <v>-3.948</v>
       </c>
       <c r="J34" s="18">
-        <v>-1.2964</v>
+        <v>-1.3</v>
       </c>
       <c r="K34" s="16">
-        <v>-4.3704000000000001</v>
+        <v>-4.37</v>
       </c>
       <c r="L34" s="13">
         <v>-1.2931999999999999</v>
@@ -3049,10 +3049,10 @@
         <v>-1.0669999999999999</v>
       </c>
       <c r="J35" s="18">
-        <v>-46.529899999999998</v>
+        <v>-46.53</v>
       </c>
       <c r="K35" s="16">
-        <v>-1.3022</v>
+        <v>-1.3</v>
       </c>
       <c r="L35" s="13">
         <v>-39.363799999999998</v>
@@ -3136,10 +3136,10 @@
         <v>0.95230000000000004</v>
       </c>
       <c r="J37" s="18">
-        <v>-1.0037</v>
+        <v>-1</v>
       </c>
       <c r="K37" s="16">
-        <v>-8.3226999999999993</v>
+        <v>-8.32</v>
       </c>
       <c r="L37" s="13">
         <v>0.95120000000000005</v>
@@ -3201,10 +3201,10 @@
         <v>0.91739999999999999</v>
       </c>
       <c r="J38" s="18">
-        <v>0.4793</v>
+        <v>0.48</v>
       </c>
       <c r="K38" s="16">
-        <v>0.83760000000000001</v>
+        <v>0.84</v>
       </c>
       <c r="L38" s="13">
         <v>0.57199999999999995</v>
@@ -3269,7 +3269,7 @@
         <v>-1.94</v>
       </c>
       <c r="K39" s="16">
-        <v>-7.2976000000000001</v>
+        <v>-7.3</v>
       </c>
       <c r="L39" s="13">
         <v>-0.2203</v>
@@ -3327,10 +3327,10 @@
         <v>0.91139999999999999</v>
       </c>
       <c r="J40" s="18">
-        <v>-0.64739999999999998</v>
+        <v>-0.65</v>
       </c>
       <c r="K40" s="16">
-        <v>0.8488</v>
+        <v>0.85</v>
       </c>
       <c r="L40" s="13">
         <v>-5.9700000000000003E-2</v>
@@ -3392,10 +3392,10 @@
         <v>0.69910000000000005</v>
       </c>
       <c r="J41" s="18">
-        <v>-1.5044999999999999</v>
+        <v>-1.5</v>
       </c>
       <c r="K41" s="16">
-        <v>0.66439999999999999</v>
+        <v>0.66</v>
       </c>
       <c r="L41" s="13">
         <v>-0.12230000000000001</v>
@@ -3457,10 +3457,10 @@
         <v>0.70730000000000004</v>
       </c>
       <c r="J42" s="18">
-        <v>-1.9440999999999999</v>
+        <v>-1.94</v>
       </c>
       <c r="K42" s="16">
-        <v>-10.667</v>
+        <v>-10.67</v>
       </c>
       <c r="L42" s="13">
         <v>-1.9684999999999999</v>
@@ -3544,10 +3544,10 @@
         <v>0.63700000000000001</v>
       </c>
       <c r="J44" s="18">
-        <v>-0.73839999999999995</v>
+        <v>-0.74</v>
       </c>
       <c r="K44" s="16">
-        <v>-1.9514</v>
+        <v>-1.95</v>
       </c>
       <c r="L44" s="13">
         <v>-1.3526</v>
@@ -3609,10 +3609,10 @@
         <v>0.89739999999999998</v>
       </c>
       <c r="J45" s="18">
-        <v>-0.78239999999999998</v>
+        <v>-0.78</v>
       </c>
       <c r="K45" s="16">
-        <v>0.9194</v>
+        <v>0.92</v>
       </c>
       <c r="L45" s="13">
         <v>-0.1305</v>
@@ -3705,11 +3705,11 @@
       </c>
       <c r="J47" s="24">
         <f t="shared" si="0"/>
-        <v>-0.28295000000000003</v>
+        <v>-0.26</v>
       </c>
       <c r="K47" s="25">
         <f t="shared" si="0"/>
-        <v>0.61945000000000006</v>
+        <v>0.64</v>
       </c>
       <c r="L47" s="26">
         <f t="shared" si="0"/>
@@ -3790,11 +3790,11 @@
       </c>
       <c r="J48" s="24">
         <f t="shared" ref="J48:Q48" si="2">MEDIAN(J24:J27,J29:J30,J32:J35)</f>
-        <v>-1.2199499999999999</v>
+        <v>-1.22</v>
       </c>
       <c r="K48" s="25">
         <f t="shared" si="2"/>
-        <v>-0.85140000000000005</v>
+        <v>-0.85000000000000009</v>
       </c>
       <c r="L48" s="26">
         <f t="shared" si="2"/>

</xml_diff>